<commit_message>
Full reset — completely fresh file
</commit_message>
<xml_diff>
--- a/finishing_data.xlsx
+++ b/finishing_data.xlsx
@@ -1,34 +1,53 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StyleDB" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BeforeWashTx" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AfterWashTx" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006A1B9A"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -43,13 +62,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -196,7 +217,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -231,7 +251,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -266,16 +285,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -397,46 +420,7 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -451,132 +435,132 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>StyleKey</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>StyleName</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ACC</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Factory</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>WashType</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>TackSample</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>StdLeadTimeHrs</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>BWWaistTie</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>BWPlacket</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>BWSleeve</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>BWBottomHem</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>BWDummy</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>BWPocket</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>BWWaistTack</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>BWTackCount</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>AWRmWashTie</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>AWRmWashTack</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>AWRmLabel</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>AWLoop</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>AWReinforce</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>AWTab</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>AWDummyRm</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>AWPocketClean</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>AWTackCount</t>
         </is>
@@ -597,102 +581,102 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>RowID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>StyleKey</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>StyleName</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Factory</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>WashType</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>TackSample</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ACC</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>InDate</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>InTime</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>InQty</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>OutDate</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>OutTime</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>OutQty</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>WIPRow</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>CumulativeWIP</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -713,102 +697,102 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>RowID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>StyleKey</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>StyleName</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Factory</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>WashType</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>TackSample</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>ACC</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>InDate</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>InTime</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>InQty</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>OutDate</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>OutTime</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>OutQty</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>WIPRow</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>CumulativeWIP</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>

</xml_diff>

<commit_message>
Force clear all data
</commit_message>
<xml_diff>
--- a/finishing_data.xlsx
+++ b/finishing_data.xlsx
@@ -1,54 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="StyleDB" sheetId="1" r:id="rId1"/>
-    <sheet name="BeforeWashTx" sheetId="2" r:id="rId2"/>
-    <sheet name="AfterWashTx" sheetId="3" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StyleDB" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BeforeWashTx" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AfterWashTx" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -67,13 +44,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -398,156 +442,143 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>RowID</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Month</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Week</v>
-      </c>
-      <c r="D1" t="str">
-        <v>StyleKey</v>
-      </c>
-      <c r="E1" t="str">
-        <v>StyleName</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Color</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Factory</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Product</v>
-      </c>
-      <c r="I1" t="str">
-        <v>WashType</v>
-      </c>
-      <c r="J1" t="str">
-        <v>TackSample</v>
-      </c>
-      <c r="K1" t="str">
-        <v>ACC</v>
-      </c>
-      <c r="L1" t="str">
-        <v>InDate</v>
-      </c>
-      <c r="M1" t="str">
-        <v>InTime</v>
-      </c>
-      <c r="N1" t="str">
-        <v>InQty</v>
-      </c>
-      <c r="O1" t="str">
-        <v>OutDate</v>
-      </c>
-      <c r="P1" t="str">
-        <v>OutTime</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>OutQty</v>
-      </c>
-      <c r="R1" t="str">
-        <v>WIPRow</v>
-      </c>
-      <c r="S1" t="str">
-        <v>CumulativeWIP</v>
-      </c>
-      <c r="T1" t="str">
-        <v>Remarks</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>1781502878597</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Jun 2026</v>
-      </c>
-      <c r="C2" t="str">
-        <v>W25</v>
-      </c>
-      <c r="D2" t="str">
-        <v>a|||pink</v>
-      </c>
-      <c r="E2" t="str">
-        <v>A</v>
-      </c>
-      <c r="F2" t="str">
-        <v>PINK</v>
-      </c>
-      <c r="G2" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Short</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Denim</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K2" t="str">
-        <v>1</v>
-      </c>
-      <c r="L2" t="str">
-        <v>2026-06-13</v>
-      </c>
-      <c r="M2" t="str">
-        <v>11:24</v>
-      </c>
-      <c r="N2">
-        <v>100</v>
-      </c>
-      <c r="O2" t="str">
-        <v>2026-06-13</v>
-      </c>
-      <c r="P2" t="str">
-        <v>16:29</v>
-      </c>
-      <c r="Q2">
-        <v>50</v>
-      </c>
-      <c r="R2">
-        <v>50</v>
-      </c>
-      <c r="S2">
-        <v>50</v>
-      </c>
-      <c r="T2" t="str">
-        <v/>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>RowID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>StyleKey</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>StyleName</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Factory</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>WashType</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>TackSample</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ACC</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>InDate</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>InTime</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>InQty</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>OutDate</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>OutTime</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>OutQty</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>WIPRow</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>CumulativeWIP</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T2"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clear all data — headers only
</commit_message>
<xml_diff>
--- a/finishing_data.xlsx
+++ b/finishing_data.xlsx
@@ -1,7 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StyleDB" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BeforeWashTx" sheetId="2" state="visible" r:id="rId2"/>
@@ -9,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyPlan" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -20,7 +25,7 @@
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -28,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -37,12 +42,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000695C"/>
+        <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="006A1B9A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000695C"/>
       </patternFill>
     </fill>
   </fills>
@@ -58,15 +68,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -213,7 +224,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -248,7 +258,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -283,16 +292,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -414,46 +427,7 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -464,136 +438,136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>StyleKey</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>StyleName</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ACC</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Factory</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>WashType</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>TackSample</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>StdLeadTimeHrs</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>BWWaistTie</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>BWPlacket</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>BWSleeve</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>BWBottomHem</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>BWDummy</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>BWPocket</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>BWWaistTack</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>BWTackCount</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>AWRmWashTie</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>AWRmWashTack</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>AWRmLabel</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>AWLoop</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>AWReinforce</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>AWTab</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>AWDummyRm</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>AWPocketClean</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>AWTackCount</t>
         </is>
@@ -601,78 +575,6 @@
       <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>MinDispatch</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>a|||black</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>BLACK</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>SGL</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Shirt</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Denim</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>2</t>
         </is>
       </c>
     </row>
@@ -687,185 +589,109 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>RowID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>StyleKey</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>StyleName</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Factory</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>WashType</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>TackSample</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ACC</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>InDate</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>InTime</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>InQty</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>OutDate</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>OutTime</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>OutQty</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>WIPRow</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>CumulativeWIP</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1781524432230</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>W25</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>a|||black</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>BLACK</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>SGL</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Shirt</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Denim</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>06:24</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>100</v>
-      </c>
-      <c r="R2" t="n">
-        <v>100</v>
-      </c>
-      <c r="S2" t="n">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -883,102 +709,102 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>RowID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>StyleKey</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>StyleName</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Factory</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>WashType</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>TackSample</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>ACC</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>InDate</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>InTime</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>InQty</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>OutDate</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>OutTime</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>OutQty</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>WIPRow</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>CumulativeWIP</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -999,32 +825,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>PlanKey</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>StyleName</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>PlanQty</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>MinDispatch</t>
         </is>

</xml_diff>

<commit_message>
Restore and fix NaN corruption — previous save wiped file
</commit_message>
<xml_diff>
--- a/finishing_data.xlsx
+++ b/finishing_data.xlsx
@@ -3317,7 +3317,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T691"/>
+  <dimension ref="A1:T684"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -45727,443 +45727,9 @@
         <v/>
       </c>
     </row>
-    <row r="685">
-      <c r="A685" t="str">
-        <v>1787204131697</v>
-      </c>
-      <c r="B685" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C685" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D685" t="str">
-        <v>m1034|||light wash</v>
-      </c>
-      <c r="E685" t="str">
-        <v>M1034</v>
-      </c>
-      <c r="F685" t="str">
-        <v>LIGHT WASH</v>
-      </c>
-      <c r="G685" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H685" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I685" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J685" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K685" t="str">
-        <v/>
-      </c>
-      <c r="L685" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M685" t="str">
-        <v>07:30</v>
-      </c>
-      <c r="N685">
-        <v>112</v>
-      </c>
-      <c r="O685" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="P685" t="str">
-        <v>15:30</v>
-      </c>
-      <c r="Q685">
-        <v>112</v>
-      </c>
-      <c r="R685">
-        <v>0</v>
-      </c>
-      <c r="S685">
-        <v>0</v>
-      </c>
-      <c r="T685" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="686">
-      <c r="A686" t="str">
-        <v>1787204164130</v>
-      </c>
-      <c r="B686" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C686" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D686" t="str">
-        <v>m1012|||brown</v>
-      </c>
-      <c r="E686" t="str">
-        <v>M1012</v>
-      </c>
-      <c r="F686" t="str">
-        <v>BROWN</v>
-      </c>
-      <c r="G686" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H686" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I686" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J686" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K686" t="str">
-        <v/>
-      </c>
-      <c r="L686" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M686" t="str">
-        <v>07:30</v>
-      </c>
-      <c r="N686">
-        <v>167</v>
-      </c>
-      <c r="O686" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="P686" t="str">
-        <v>03:30</v>
-      </c>
-      <c r="Q686">
-        <v>167</v>
-      </c>
-      <c r="R686">
-        <v>0</v>
-      </c>
-      <c r="S686">
-        <v>0</v>
-      </c>
-      <c r="T686" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="687">
-      <c r="A687" t="str">
-        <v>1787204191482</v>
-      </c>
-      <c r="B687" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C687" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D687" t="str">
-        <v>m1026|||olive green</v>
-      </c>
-      <c r="E687" t="str">
-        <v>M1026</v>
-      </c>
-      <c r="F687" t="str">
-        <v>OLIVE GREEN</v>
-      </c>
-      <c r="G687" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H687" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I687" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J687" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K687" t="str">
-        <v/>
-      </c>
-      <c r="L687" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M687" t="str">
-        <v>07:30</v>
-      </c>
-      <c r="N687">
-        <v>228</v>
-      </c>
-      <c r="O687" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="P687" t="str">
-        <v>15:30</v>
-      </c>
-      <c r="Q687">
-        <v>228</v>
-      </c>
-      <c r="R687">
-        <v>0</v>
-      </c>
-      <c r="S687">
-        <v>0</v>
-      </c>
-      <c r="T687" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="688">
-      <c r="A688" t="str">
-        <v>1787204222642</v>
-      </c>
-      <c r="B688" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C688" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D688" t="str">
-        <v>m1034|||light wash</v>
-      </c>
-      <c r="E688" t="str">
-        <v>M1034</v>
-      </c>
-      <c r="F688" t="str">
-        <v>LIGHT WASH</v>
-      </c>
-      <c r="G688" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H688" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I688" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J688" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K688" t="str">
-        <v/>
-      </c>
-      <c r="L688" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M688" t="str">
-        <v>07:30</v>
-      </c>
-      <c r="N688">
-        <v>96</v>
-      </c>
-      <c r="O688" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="P688" t="str">
-        <v>15:30</v>
-      </c>
-      <c r="Q688">
-        <v>96</v>
-      </c>
-      <c r="R688">
-        <v>0</v>
-      </c>
-      <c r="S688">
-        <v>0</v>
-      </c>
-      <c r="T688" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="689">
-      <c r="A689" t="str">
-        <v>1787204287899</v>
-      </c>
-      <c r="B689" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C689" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D689" t="str">
-        <v>m1026|||brown</v>
-      </c>
-      <c r="E689" t="str">
-        <v>M1026</v>
-      </c>
-      <c r="F689" t="str">
-        <v>BROWN</v>
-      </c>
-      <c r="G689" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H689" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I689" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J689" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K689" t="str">
-        <v/>
-      </c>
-      <c r="L689" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M689" t="str">
-        <v>07:30</v>
-      </c>
-      <c r="N689">
-        <v>16</v>
-      </c>
-      <c r="O689" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="P689" t="str">
-        <v>15:30</v>
-      </c>
-      <c r="Q689">
-        <v>16</v>
-      </c>
-      <c r="R689">
-        <v>0</v>
-      </c>
-      <c r="S689">
-        <v>0</v>
-      </c>
-      <c r="T689" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="690">
-      <c r="A690" t="str">
-        <v>1787204316787</v>
-      </c>
-      <c r="B690" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C690" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D690" t="str">
-        <v>m1012|||washed black</v>
-      </c>
-      <c r="E690" t="str">
-        <v>M1012</v>
-      </c>
-      <c r="F690" t="str">
-        <v>WASHED BLACK</v>
-      </c>
-      <c r="G690" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H690" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I690" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J690" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K690" t="str">
-        <v/>
-      </c>
-      <c r="L690" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M690" t="str">
-        <v>07:30</v>
-      </c>
-      <c r="N690">
-        <v>9</v>
-      </c>
-      <c r="O690" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="P690" t="str">
-        <v>15:30</v>
-      </c>
-      <c r="Q690">
-        <v>9</v>
-      </c>
-      <c r="R690">
-        <v>0</v>
-      </c>
-      <c r="S690">
-        <v>0</v>
-      </c>
-      <c r="T690" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="691">
-      <c r="A691" t="str">
-        <v>1787204344971</v>
-      </c>
-      <c r="B691" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C691" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D691" t="str">
-        <v>m1012|||washed black</v>
-      </c>
-      <c r="E691" t="str">
-        <v>M1012</v>
-      </c>
-      <c r="F691" t="str">
-        <v>WASHED BLACK</v>
-      </c>
-      <c r="G691" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H691" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I691" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J691" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K691" t="str">
-        <v/>
-      </c>
-      <c r="L691" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M691" t="str">
-        <v>07:30</v>
-      </c>
-      <c r="N691">
-        <v>187</v>
-      </c>
-      <c r="O691" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="P691" t="str">
-        <v>15:30</v>
-      </c>
-      <c r="Q691">
-        <v>187</v>
-      </c>
-      <c r="R691">
-        <v>0</v>
-      </c>
-      <c r="S691">
-        <v>0</v>
-      </c>
-      <c r="T691" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T691"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T684"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -90267,22 +89833,22 @@
         <v>0</v>
       </c>
       <c r="L2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="Q2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="R2" t="str">
         <v>0</v>

</xml_diff>

<commit_message>
Emergency restore — client still using old app
</commit_message>
<xml_diff>
--- a/finishing_data.xlsx
+++ b/finishing_data.xlsx
@@ -515,13 +515,13 @@
         <v/>
       </c>
       <c r="J2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K2" t="str">
         <v>No</v>
       </c>
-      <c r="K2" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L2" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M2" t="str">
         <v>No</v>
@@ -530,11 +530,11 @@
         <v>No</v>
       </c>
       <c r="O2" t="str">
+        <v>No</v>
+      </c>
+      <c r="P2" t="str">
         <v>3</v>
       </c>
-      <c r="P2" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q2" t="str">
         <v>Yes</v>
       </c>
@@ -548,19 +548,19 @@
         <v>Yes</v>
       </c>
       <c r="U2" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V2" t="str">
         <v>No</v>
       </c>
       <c r="W2" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y2" t="str">
         <v>6</v>
-      </c>
-      <c r="Y2" t="str">
-        <v>0</v>
       </c>
       <c r="Z2" t="str">
         <v>0</v>
@@ -598,13 +598,13 @@
         <v/>
       </c>
       <c r="J3" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K3" t="str">
         <v>No</v>
       </c>
-      <c r="K3" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L3" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M3" t="str">
         <v>No</v>
@@ -613,11 +613,11 @@
         <v>No</v>
       </c>
       <c r="O3" t="str">
+        <v>No</v>
+      </c>
+      <c r="P3" t="str">
         <v>3</v>
       </c>
-      <c r="P3" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q3" t="str">
         <v>Yes</v>
       </c>
@@ -631,19 +631,19 @@
         <v>Yes</v>
       </c>
       <c r="U3" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V3" t="str">
         <v>No</v>
       </c>
       <c r="W3" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X3" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y3" t="str">
         <v>6</v>
-      </c>
-      <c r="Y3" t="str">
-        <v>0</v>
       </c>
       <c r="Z3" t="str">
         <v>0</v>
@@ -681,13 +681,13 @@
         <v/>
       </c>
       <c r="J4" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K4" t="str">
         <v>No</v>
       </c>
-      <c r="K4" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L4" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M4" t="str">
         <v>No</v>
@@ -696,11 +696,11 @@
         <v>No</v>
       </c>
       <c r="O4" t="str">
+        <v>No</v>
+      </c>
+      <c r="P4" t="str">
         <v>3</v>
       </c>
-      <c r="P4" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q4" t="str">
         <v>Yes</v>
       </c>
@@ -714,19 +714,19 @@
         <v>Yes</v>
       </c>
       <c r="U4" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V4" t="str">
         <v>No</v>
       </c>
       <c r="W4" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X4" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y4" t="str">
         <v>6</v>
-      </c>
-      <c r="Y4" t="str">
-        <v>0</v>
       </c>
       <c r="Z4" t="str">
         <v>0</v>
@@ -764,13 +764,13 @@
         <v/>
       </c>
       <c r="J5" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K5" t="str">
         <v>No</v>
       </c>
-      <c r="K5" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L5" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M5" t="str">
         <v>No</v>
@@ -779,11 +779,11 @@
         <v>No</v>
       </c>
       <c r="O5" t="str">
+        <v>No</v>
+      </c>
+      <c r="P5" t="str">
         <v>3</v>
       </c>
-      <c r="P5" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q5" t="str">
         <v>Yes</v>
       </c>
@@ -797,19 +797,19 @@
         <v>Yes</v>
       </c>
       <c r="U5" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V5" t="str">
         <v>No</v>
       </c>
       <c r="W5" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X5" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y5" t="str">
         <v>6</v>
-      </c>
-      <c r="Y5" t="str">
-        <v>0</v>
       </c>
       <c r="Z5" t="str">
         <v>0</v>
@@ -847,13 +847,13 @@
         <v/>
       </c>
       <c r="J6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K6" t="str">
         <v>No</v>
       </c>
-      <c r="K6" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L6" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M6" t="str">
         <v>No</v>
@@ -862,11 +862,11 @@
         <v>No</v>
       </c>
       <c r="O6" t="str">
+        <v>No</v>
+      </c>
+      <c r="P6" t="str">
         <v>3</v>
       </c>
-      <c r="P6" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q6" t="str">
         <v>Yes</v>
       </c>
@@ -880,19 +880,19 @@
         <v>Yes</v>
       </c>
       <c r="U6" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V6" t="str">
         <v>No</v>
       </c>
       <c r="W6" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y6" t="str">
         <v>6</v>
-      </c>
-      <c r="Y6" t="str">
-        <v>0</v>
       </c>
       <c r="Z6" t="str">
         <v>0</v>
@@ -930,13 +930,13 @@
         <v/>
       </c>
       <c r="J7" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K7" t="str">
         <v>No</v>
       </c>
-      <c r="K7" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L7" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M7" t="str">
         <v>No</v>
@@ -945,11 +945,11 @@
         <v>No</v>
       </c>
       <c r="O7" t="str">
+        <v>No</v>
+      </c>
+      <c r="P7" t="str">
         <v>3</v>
       </c>
-      <c r="P7" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q7" t="str">
         <v>Yes</v>
       </c>
@@ -963,19 +963,19 @@
         <v>Yes</v>
       </c>
       <c r="U7" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V7" t="str">
         <v>No</v>
       </c>
       <c r="W7" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X7" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y7" t="str">
         <v>6</v>
-      </c>
-      <c r="Y7" t="str">
-        <v>0</v>
       </c>
       <c r="Z7" t="str">
         <v>0</v>
@@ -1013,13 +1013,13 @@
         <v/>
       </c>
       <c r="J8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K8" t="str">
         <v>No</v>
       </c>
-      <c r="K8" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L8" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M8" t="str">
         <v>No</v>
@@ -1028,11 +1028,11 @@
         <v>No</v>
       </c>
       <c r="O8" t="str">
+        <v>No</v>
+      </c>
+      <c r="P8" t="str">
         <v>3</v>
       </c>
-      <c r="P8" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q8" t="str">
         <v>Yes</v>
       </c>
@@ -1046,19 +1046,19 @@
         <v>Yes</v>
       </c>
       <c r="U8" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V8" t="str">
         <v>No</v>
       </c>
       <c r="W8" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y8" t="str">
         <v>6</v>
-      </c>
-      <c r="Y8" t="str">
-        <v>0</v>
       </c>
       <c r="Z8" t="str">
         <v>0</v>
@@ -1096,13 +1096,13 @@
         <v/>
       </c>
       <c r="J9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K9" t="str">
         <v>No</v>
       </c>
-      <c r="K9" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L9" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M9" t="str">
         <v>No</v>
@@ -1111,11 +1111,11 @@
         <v>No</v>
       </c>
       <c r="O9" t="str">
+        <v>No</v>
+      </c>
+      <c r="P9" t="str">
         <v>3</v>
       </c>
-      <c r="P9" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q9" t="str">
         <v>Yes</v>
       </c>
@@ -1129,19 +1129,19 @@
         <v>Yes</v>
       </c>
       <c r="U9" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V9" t="str">
         <v>No</v>
       </c>
       <c r="W9" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y9" t="str">
         <v>6</v>
-      </c>
-      <c r="Y9" t="str">
-        <v>0</v>
       </c>
       <c r="Z9" t="str">
         <v>0</v>
@@ -1179,13 +1179,13 @@
         <v/>
       </c>
       <c r="J10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K10" t="str">
         <v>No</v>
       </c>
-      <c r="K10" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L10" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M10" t="str">
         <v>No</v>
@@ -1194,11 +1194,11 @@
         <v>No</v>
       </c>
       <c r="O10" t="str">
+        <v>No</v>
+      </c>
+      <c r="P10" t="str">
         <v>3</v>
       </c>
-      <c r="P10" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q10" t="str">
         <v>Yes</v>
       </c>
@@ -1212,19 +1212,19 @@
         <v>Yes</v>
       </c>
       <c r="U10" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V10" t="str">
         <v>No</v>
       </c>
       <c r="W10" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y10" t="str">
         <v>6</v>
-      </c>
-      <c r="Y10" t="str">
-        <v>0</v>
       </c>
       <c r="Z10" t="str">
         <v>0</v>
@@ -1262,13 +1262,13 @@
         <v/>
       </c>
       <c r="J11" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K11" t="str">
         <v>No</v>
       </c>
-      <c r="K11" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L11" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M11" t="str">
         <v>No</v>
@@ -1277,11 +1277,11 @@
         <v>No</v>
       </c>
       <c r="O11" t="str">
+        <v>No</v>
+      </c>
+      <c r="P11" t="str">
         <v>3</v>
       </c>
-      <c r="P11" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q11" t="str">
         <v>Yes</v>
       </c>
@@ -1295,19 +1295,19 @@
         <v>Yes</v>
       </c>
       <c r="U11" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V11" t="str">
         <v>No</v>
       </c>
       <c r="W11" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X11" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y11" t="str">
         <v>6</v>
-      </c>
-      <c r="Y11" t="str">
-        <v>0</v>
       </c>
       <c r="Z11" t="str">
         <v>0</v>
@@ -1345,13 +1345,13 @@
         <v/>
       </c>
       <c r="J12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K12" t="str">
         <v>No</v>
       </c>
-      <c r="K12" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L12" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M12" t="str">
         <v>No</v>
@@ -1360,11 +1360,11 @@
         <v>No</v>
       </c>
       <c r="O12" t="str">
+        <v>No</v>
+      </c>
+      <c r="P12" t="str">
         <v>3</v>
       </c>
-      <c r="P12" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q12" t="str">
         <v>Yes</v>
       </c>
@@ -1378,19 +1378,19 @@
         <v>Yes</v>
       </c>
       <c r="U12" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V12" t="str">
         <v>No</v>
       </c>
       <c r="W12" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y12" t="str">
         <v>6</v>
-      </c>
-      <c r="Y12" t="str">
-        <v>0</v>
       </c>
       <c r="Z12" t="str">
         <v>0</v>
@@ -1428,13 +1428,13 @@
         <v/>
       </c>
       <c r="J13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K13" t="str">
         <v>No</v>
       </c>
-      <c r="K13" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L13" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M13" t="str">
         <v>No</v>
@@ -1443,11 +1443,11 @@
         <v>No</v>
       </c>
       <c r="O13" t="str">
+        <v>No</v>
+      </c>
+      <c r="P13" t="str">
         <v>3</v>
       </c>
-      <c r="P13" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q13" t="str">
         <v>Yes</v>
       </c>
@@ -1461,19 +1461,19 @@
         <v>Yes</v>
       </c>
       <c r="U13" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V13" t="str">
         <v>No</v>
       </c>
       <c r="W13" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y13" t="str">
         <v>6</v>
-      </c>
-      <c r="Y13" t="str">
-        <v>0</v>
       </c>
       <c r="Z13" t="str">
         <v>0</v>
@@ -1511,13 +1511,13 @@
         <v/>
       </c>
       <c r="J14" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K14" t="str">
         <v>No</v>
       </c>
-      <c r="K14" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L14" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M14" t="str">
         <v>No</v>
@@ -1526,11 +1526,11 @@
         <v>No</v>
       </c>
       <c r="O14" t="str">
+        <v>No</v>
+      </c>
+      <c r="P14" t="str">
         <v>3</v>
       </c>
-      <c r="P14" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q14" t="str">
         <v>Yes</v>
       </c>
@@ -1544,19 +1544,19 @@
         <v>Yes</v>
       </c>
       <c r="U14" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V14" t="str">
         <v>No</v>
       </c>
       <c r="W14" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X14" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y14" t="str">
         <v>6</v>
-      </c>
-      <c r="Y14" t="str">
-        <v>0</v>
       </c>
       <c r="Z14" t="str">
         <v>0</v>
@@ -1594,13 +1594,13 @@
         <v/>
       </c>
       <c r="J15" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K15" t="str">
         <v>No</v>
       </c>
-      <c r="K15" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L15" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M15" t="str">
         <v>No</v>
@@ -1609,11 +1609,11 @@
         <v>No</v>
       </c>
       <c r="O15" t="str">
+        <v>No</v>
+      </c>
+      <c r="P15" t="str">
         <v>3</v>
       </c>
-      <c r="P15" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q15" t="str">
         <v>Yes</v>
       </c>
@@ -1627,19 +1627,19 @@
         <v>Yes</v>
       </c>
       <c r="U15" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V15" t="str">
         <v>No</v>
       </c>
       <c r="W15" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X15" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y15" t="str">
         <v>6</v>
-      </c>
-      <c r="Y15" t="str">
-        <v>0</v>
       </c>
       <c r="Z15" t="str">
         <v>0</v>
@@ -1677,13 +1677,13 @@
         <v/>
       </c>
       <c r="J16" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K16" t="str">
         <v>No</v>
       </c>
-      <c r="K16" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L16" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M16" t="str">
         <v>No</v>
@@ -1692,11 +1692,11 @@
         <v>No</v>
       </c>
       <c r="O16" t="str">
+        <v>No</v>
+      </c>
+      <c r="P16" t="str">
         <v>3</v>
       </c>
-      <c r="P16" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q16" t="str">
         <v>Yes</v>
       </c>
@@ -1710,19 +1710,19 @@
         <v>Yes</v>
       </c>
       <c r="U16" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V16" t="str">
         <v>No</v>
       </c>
       <c r="W16" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X16" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y16" t="str">
         <v>6</v>
-      </c>
-      <c r="Y16" t="str">
-        <v>0</v>
       </c>
       <c r="Z16" t="str">
         <v>0</v>
@@ -1760,13 +1760,13 @@
         <v/>
       </c>
       <c r="J17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K17" t="str">
         <v>No</v>
       </c>
-      <c r="K17" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L17" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M17" t="str">
         <v>No</v>
@@ -1775,11 +1775,11 @@
         <v>No</v>
       </c>
       <c r="O17" t="str">
+        <v>No</v>
+      </c>
+      <c r="P17" t="str">
         <v>3</v>
       </c>
-      <c r="P17" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q17" t="str">
         <v>Yes</v>
       </c>
@@ -1793,19 +1793,19 @@
         <v>Yes</v>
       </c>
       <c r="U17" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V17" t="str">
         <v>No</v>
       </c>
       <c r="W17" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y17" t="str">
         <v>6</v>
-      </c>
-      <c r="Y17" t="str">
-        <v>0</v>
       </c>
       <c r="Z17" t="str">
         <v>0</v>
@@ -1843,13 +1843,13 @@
         <v/>
       </c>
       <c r="J18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K18" t="str">
         <v>No</v>
       </c>
-      <c r="K18" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L18" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M18" t="str">
         <v>No</v>
@@ -1858,11 +1858,11 @@
         <v>No</v>
       </c>
       <c r="O18" t="str">
+        <v>No</v>
+      </c>
+      <c r="P18" t="str">
         <v>3</v>
       </c>
-      <c r="P18" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q18" t="str">
         <v>Yes</v>
       </c>
@@ -1876,19 +1876,19 @@
         <v>Yes</v>
       </c>
       <c r="U18" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V18" t="str">
         <v>No</v>
       </c>
       <c r="W18" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y18" t="str">
         <v>6</v>
-      </c>
-      <c r="Y18" t="str">
-        <v>0</v>
       </c>
       <c r="Z18" t="str">
         <v>0</v>
@@ -1926,13 +1926,13 @@
         <v/>
       </c>
       <c r="J19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K19" t="str">
         <v>No</v>
       </c>
-      <c r="K19" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L19" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M19" t="str">
         <v>No</v>
@@ -1941,11 +1941,11 @@
         <v>No</v>
       </c>
       <c r="O19" t="str">
+        <v>No</v>
+      </c>
+      <c r="P19" t="str">
         <v>3</v>
       </c>
-      <c r="P19" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q19" t="str">
         <v>Yes</v>
       </c>
@@ -1959,19 +1959,19 @@
         <v>Yes</v>
       </c>
       <c r="U19" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V19" t="str">
         <v>No</v>
       </c>
       <c r="W19" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y19" t="str">
         <v>6</v>
-      </c>
-      <c r="Y19" t="str">
-        <v>0</v>
       </c>
       <c r="Z19" t="str">
         <v>0</v>
@@ -2009,13 +2009,13 @@
         <v/>
       </c>
       <c r="J20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K20" t="str">
         <v>No</v>
       </c>
-      <c r="K20" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L20" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M20" t="str">
         <v>No</v>
@@ -2024,11 +2024,11 @@
         <v>No</v>
       </c>
       <c r="O20" t="str">
+        <v>No</v>
+      </c>
+      <c r="P20" t="str">
         <v>3</v>
       </c>
-      <c r="P20" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q20" t="str">
         <v>Yes</v>
       </c>
@@ -2042,19 +2042,19 @@
         <v>Yes</v>
       </c>
       <c r="U20" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V20" t="str">
         <v>No</v>
       </c>
       <c r="W20" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y20" t="str">
         <v>6</v>
-      </c>
-      <c r="Y20" t="str">
-        <v>0</v>
       </c>
       <c r="Z20" t="str">
         <v>0</v>
@@ -2092,13 +2092,13 @@
         <v/>
       </c>
       <c r="J21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K21" t="str">
         <v>No</v>
       </c>
-      <c r="K21" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L21" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M21" t="str">
         <v>No</v>
@@ -2107,11 +2107,11 @@
         <v>No</v>
       </c>
       <c r="O21" t="str">
+        <v>No</v>
+      </c>
+      <c r="P21" t="str">
         <v>3</v>
       </c>
-      <c r="P21" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q21" t="str">
         <v>Yes</v>
       </c>
@@ -2125,19 +2125,19 @@
         <v>Yes</v>
       </c>
       <c r="U21" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V21" t="str">
         <v>No</v>
       </c>
       <c r="W21" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y21" t="str">
         <v>6</v>
-      </c>
-      <c r="Y21" t="str">
-        <v>0</v>
       </c>
       <c r="Z21" t="str">
         <v>0</v>
@@ -2175,13 +2175,13 @@
         <v/>
       </c>
       <c r="J22" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K22" t="str">
         <v>No</v>
       </c>
-      <c r="K22" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L22" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M22" t="str">
         <v>No</v>
@@ -2190,11 +2190,11 @@
         <v>No</v>
       </c>
       <c r="O22" t="str">
+        <v>No</v>
+      </c>
+      <c r="P22" t="str">
         <v>3</v>
       </c>
-      <c r="P22" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q22" t="str">
         <v>Yes</v>
       </c>
@@ -2208,19 +2208,19 @@
         <v>Yes</v>
       </c>
       <c r="U22" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V22" t="str">
         <v>No</v>
       </c>
       <c r="W22" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X22" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y22" t="str">
         <v>6</v>
-      </c>
-      <c r="Y22" t="str">
-        <v>0</v>
       </c>
       <c r="Z22" t="str">
         <v>0</v>
@@ -2258,13 +2258,13 @@
         <v/>
       </c>
       <c r="J23" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K23" t="str">
         <v>No</v>
       </c>
-      <c r="K23" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L23" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M23" t="str">
         <v>No</v>
@@ -2273,11 +2273,11 @@
         <v>No</v>
       </c>
       <c r="O23" t="str">
+        <v>No</v>
+      </c>
+      <c r="P23" t="str">
         <v>3</v>
       </c>
-      <c r="P23" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q23" t="str">
         <v>Yes</v>
       </c>
@@ -2291,19 +2291,19 @@
         <v>Yes</v>
       </c>
       <c r="U23" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V23" t="str">
         <v>No</v>
       </c>
       <c r="W23" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X23" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y23" t="str">
         <v>6</v>
-      </c>
-      <c r="Y23" t="str">
-        <v>0</v>
       </c>
       <c r="Z23" t="str">
         <v>0</v>
@@ -2341,13 +2341,13 @@
         <v/>
       </c>
       <c r="J24" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K24" t="str">
         <v>No</v>
       </c>
-      <c r="K24" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L24" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M24" t="str">
         <v>No</v>
@@ -2356,11 +2356,11 @@
         <v>No</v>
       </c>
       <c r="O24" t="str">
+        <v>No</v>
+      </c>
+      <c r="P24" t="str">
         <v>3</v>
       </c>
-      <c r="P24" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q24" t="str">
         <v>Yes</v>
       </c>
@@ -2374,19 +2374,19 @@
         <v>Yes</v>
       </c>
       <c r="U24" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V24" t="str">
         <v>No</v>
       </c>
       <c r="W24" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X24" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y24" t="str">
         <v>6</v>
-      </c>
-      <c r="Y24" t="str">
-        <v>0</v>
       </c>
       <c r="Z24" t="str">
         <v>0</v>
@@ -2424,13 +2424,13 @@
         <v/>
       </c>
       <c r="J25" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K25" t="str">
         <v>No</v>
       </c>
-      <c r="K25" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L25" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M25" t="str">
         <v>No</v>
@@ -2439,11 +2439,11 @@
         <v>No</v>
       </c>
       <c r="O25" t="str">
+        <v>No</v>
+      </c>
+      <c r="P25" t="str">
         <v>3</v>
       </c>
-      <c r="P25" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q25" t="str">
         <v>Yes</v>
       </c>
@@ -2457,19 +2457,19 @@
         <v>Yes</v>
       </c>
       <c r="U25" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V25" t="str">
         <v>No</v>
       </c>
       <c r="W25" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X25" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y25" t="str">
         <v>6</v>
-      </c>
-      <c r="Y25" t="str">
-        <v>0</v>
       </c>
       <c r="Z25" t="str">
         <v>0</v>
@@ -2507,13 +2507,13 @@
         <v/>
       </c>
       <c r="J26" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K26" t="str">
         <v>No</v>
       </c>
-      <c r="K26" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L26" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M26" t="str">
         <v>No</v>
@@ -2522,11 +2522,11 @@
         <v>No</v>
       </c>
       <c r="O26" t="str">
+        <v>No</v>
+      </c>
+      <c r="P26" t="str">
         <v>3</v>
       </c>
-      <c r="P26" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q26" t="str">
         <v>Yes</v>
       </c>
@@ -2540,19 +2540,19 @@
         <v>Yes</v>
       </c>
       <c r="U26" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V26" t="str">
         <v>No</v>
       </c>
       <c r="W26" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X26" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y26" t="str">
         <v>6</v>
-      </c>
-      <c r="Y26" t="str">
-        <v>0</v>
       </c>
       <c r="Z26" t="str">
         <v>0</v>
@@ -2590,13 +2590,13 @@
         <v/>
       </c>
       <c r="J27" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K27" t="str">
         <v>No</v>
       </c>
-      <c r="K27" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L27" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M27" t="str">
         <v>No</v>
@@ -2605,11 +2605,11 @@
         <v>No</v>
       </c>
       <c r="O27" t="str">
+        <v>No</v>
+      </c>
+      <c r="P27" t="str">
         <v>3</v>
       </c>
-      <c r="P27" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q27" t="str">
         <v>Yes</v>
       </c>
@@ -2623,19 +2623,19 @@
         <v>Yes</v>
       </c>
       <c r="U27" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V27" t="str">
         <v>No</v>
       </c>
       <c r="W27" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X27" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y27" t="str">
         <v>6</v>
-      </c>
-      <c r="Y27" t="str">
-        <v>0</v>
       </c>
       <c r="Z27" t="str">
         <v>0</v>
@@ -2673,13 +2673,13 @@
         <v/>
       </c>
       <c r="J28" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K28" t="str">
         <v>No</v>
       </c>
-      <c r="K28" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L28" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M28" t="str">
         <v>No</v>
@@ -2688,11 +2688,11 @@
         <v>No</v>
       </c>
       <c r="O28" t="str">
+        <v>No</v>
+      </c>
+      <c r="P28" t="str">
         <v>3</v>
       </c>
-      <c r="P28" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q28" t="str">
         <v>Yes</v>
       </c>
@@ -2706,19 +2706,19 @@
         <v>Yes</v>
       </c>
       <c r="U28" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V28" t="str">
         <v>No</v>
       </c>
       <c r="W28" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X28" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y28" t="str">
         <v>6</v>
-      </c>
-      <c r="Y28" t="str">
-        <v>0</v>
       </c>
       <c r="Z28" t="str">
         <v>0</v>
@@ -2756,13 +2756,13 @@
         <v/>
       </c>
       <c r="J29" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K29" t="str">
         <v>No</v>
       </c>
-      <c r="K29" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L29" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M29" t="str">
         <v>No</v>
@@ -2771,11 +2771,11 @@
         <v>No</v>
       </c>
       <c r="O29" t="str">
+        <v>No</v>
+      </c>
+      <c r="P29" t="str">
         <v>3</v>
       </c>
-      <c r="P29" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q29" t="str">
         <v>Yes</v>
       </c>
@@ -2789,19 +2789,19 @@
         <v>Yes</v>
       </c>
       <c r="U29" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V29" t="str">
         <v>No</v>
       </c>
       <c r="W29" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X29" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y29" t="str">
         <v>6</v>
-      </c>
-      <c r="Y29" t="str">
-        <v>0</v>
       </c>
       <c r="Z29" t="str">
         <v>0</v>
@@ -2839,13 +2839,13 @@
         <v/>
       </c>
       <c r="J30" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K30" t="str">
         <v>No</v>
       </c>
-      <c r="K30" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L30" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M30" t="str">
         <v>No</v>
@@ -2854,11 +2854,11 @@
         <v>No</v>
       </c>
       <c r="O30" t="str">
+        <v>No</v>
+      </c>
+      <c r="P30" t="str">
         <v>3</v>
       </c>
-      <c r="P30" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q30" t="str">
         <v>Yes</v>
       </c>
@@ -2872,19 +2872,19 @@
         <v>Yes</v>
       </c>
       <c r="U30" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V30" t="str">
         <v>No</v>
       </c>
       <c r="W30" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X30" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y30" t="str">
         <v>6</v>
-      </c>
-      <c r="Y30" t="str">
-        <v>0</v>
       </c>
       <c r="Z30" t="str">
         <v>0</v>
@@ -2922,13 +2922,13 @@
         <v/>
       </c>
       <c r="J31" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K31" t="str">
         <v>No</v>
       </c>
-      <c r="K31" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L31" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M31" t="str">
         <v>No</v>
@@ -2937,11 +2937,11 @@
         <v>No</v>
       </c>
       <c r="O31" t="str">
+        <v>No</v>
+      </c>
+      <c r="P31" t="str">
         <v>3</v>
       </c>
-      <c r="P31" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q31" t="str">
         <v>Yes</v>
       </c>
@@ -2955,19 +2955,19 @@
         <v>Yes</v>
       </c>
       <c r="U31" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V31" t="str">
         <v>No</v>
       </c>
       <c r="W31" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X31" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y31" t="str">
         <v>6</v>
-      </c>
-      <c r="Y31" t="str">
-        <v>0</v>
       </c>
       <c r="Z31" t="str">
         <v>0</v>
@@ -3005,13 +3005,13 @@
         <v/>
       </c>
       <c r="J32" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K32" t="str">
         <v>No</v>
       </c>
-      <c r="K32" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L32" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M32" t="str">
         <v>No</v>
@@ -3020,11 +3020,11 @@
         <v>No</v>
       </c>
       <c r="O32" t="str">
+        <v>No</v>
+      </c>
+      <c r="P32" t="str">
         <v>3</v>
       </c>
-      <c r="P32" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q32" t="str">
         <v>Yes</v>
       </c>
@@ -3038,19 +3038,19 @@
         <v>Yes</v>
       </c>
       <c r="U32" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V32" t="str">
         <v>No</v>
       </c>
       <c r="W32" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X32" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y32" t="str">
         <v>6</v>
-      </c>
-      <c r="Y32" t="str">
-        <v>0</v>
       </c>
       <c r="Z32" t="str">
         <v>0</v>
@@ -3088,13 +3088,13 @@
         <v/>
       </c>
       <c r="J33" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K33" t="str">
         <v>No</v>
       </c>
-      <c r="K33" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L33" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M33" t="str">
         <v>No</v>
@@ -3103,11 +3103,11 @@
         <v>No</v>
       </c>
       <c r="O33" t="str">
+        <v>No</v>
+      </c>
+      <c r="P33" t="str">
         <v>3</v>
       </c>
-      <c r="P33" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q33" t="str">
         <v>Yes</v>
       </c>
@@ -3121,19 +3121,19 @@
         <v>Yes</v>
       </c>
       <c r="U33" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V33" t="str">
         <v>No</v>
       </c>
       <c r="W33" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X33" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y33" t="str">
         <v>6</v>
-      </c>
-      <c r="Y33" t="str">
-        <v>0</v>
       </c>
       <c r="Z33" t="str">
         <v>0</v>
@@ -3171,13 +3171,13 @@
         <v/>
       </c>
       <c r="J34" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K34" t="str">
         <v>No</v>
       </c>
-      <c r="K34" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L34" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M34" t="str">
         <v>No</v>
@@ -3186,11 +3186,11 @@
         <v>No</v>
       </c>
       <c r="O34" t="str">
+        <v>No</v>
+      </c>
+      <c r="P34" t="str">
         <v>3</v>
       </c>
-      <c r="P34" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q34" t="str">
         <v>Yes</v>
       </c>
@@ -3204,19 +3204,19 @@
         <v>Yes</v>
       </c>
       <c r="U34" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V34" t="str">
         <v>No</v>
       </c>
       <c r="W34" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X34" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y34" t="str">
         <v>6</v>
-      </c>
-      <c r="Y34" t="str">
-        <v>0</v>
       </c>
       <c r="Z34" t="str">
         <v>0</v>
@@ -3254,13 +3254,13 @@
         <v/>
       </c>
       <c r="J35" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K35" t="str">
         <v>No</v>
       </c>
-      <c r="K35" t="str">
-        <v>Yes</v>
-      </c>
       <c r="L35" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="M35" t="str">
         <v>No</v>
@@ -3269,11 +3269,11 @@
         <v>No</v>
       </c>
       <c r="O35" t="str">
+        <v>No</v>
+      </c>
+      <c r="P35" t="str">
         <v>3</v>
       </c>
-      <c r="P35" t="str">
-        <v>Yes</v>
-      </c>
       <c r="Q35" t="str">
         <v>Yes</v>
       </c>
@@ -3287,19 +3287,19 @@
         <v>Yes</v>
       </c>
       <c r="U35" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="V35" t="str">
         <v>No</v>
       </c>
       <c r="W35" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="X35" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Y35" t="str">
         <v>6</v>
-      </c>
-      <c r="Y35" t="str">
-        <v>0</v>
       </c>
       <c r="Z35" t="str">
         <v>0</v>
@@ -3317,7 +3317,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T703"/>
+  <dimension ref="A1:T684"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -45727,1187 +45727,9 @@
         <v/>
       </c>
     </row>
-    <row r="685">
-      <c r="A685" t="str">
-        <v>1787221266742</v>
-      </c>
-      <c r="B685" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C685" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D685" t="str">
-        <v>m1026|||brown</v>
-      </c>
-      <c r="E685" t="str">
-        <v>M1026</v>
-      </c>
-      <c r="F685" t="str">
-        <v>BROWN</v>
-      </c>
-      <c r="G685" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H685" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I685" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J685" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K685" t="str">
-        <v/>
-      </c>
-      <c r="L685" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M685" t="str">
-        <v>07:49</v>
-      </c>
-      <c r="N685">
-        <v>8</v>
-      </c>
-      <c r="O685" t="str">
-        <v/>
-      </c>
-      <c r="P685" t="str">
-        <v/>
-      </c>
-      <c r="Q685" t="str">
-        <v/>
-      </c>
-      <c r="R685">
-        <v>8</v>
-      </c>
-      <c r="S685">
-        <v>8</v>
-      </c>
-      <c r="T685" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="686">
-      <c r="A686" t="str">
-        <v>1787221366463</v>
-      </c>
-      <c r="B686" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C686" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D686" t="str">
-        <v>m1012|||washed black</v>
-      </c>
-      <c r="E686" t="str">
-        <v>M1012</v>
-      </c>
-      <c r="F686" t="str">
-        <v>WASHED BLACK</v>
-      </c>
-      <c r="G686" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H686" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I686" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J686" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K686" t="str">
-        <v/>
-      </c>
-      <c r="L686" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M686" t="str">
-        <v>07:51</v>
-      </c>
-      <c r="N686">
-        <v>434</v>
-      </c>
-      <c r="O686" t="str">
-        <v/>
-      </c>
-      <c r="P686" t="str">
-        <v/>
-      </c>
-      <c r="Q686" t="str">
-        <v/>
-      </c>
-      <c r="R686">
-        <v>434</v>
-      </c>
-      <c r="S686">
-        <v>434</v>
-      </c>
-      <c r="T686" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="687">
-      <c r="A687" t="str">
-        <v>1787221445440</v>
-      </c>
-      <c r="B687" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C687" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D687" t="str">
-        <v>m1034|||light wash</v>
-      </c>
-      <c r="E687" t="str">
-        <v>M1034</v>
-      </c>
-      <c r="F687" t="str">
-        <v>LIGHT WASH</v>
-      </c>
-      <c r="G687" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H687" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I687" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J687" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K687" t="str">
-        <v/>
-      </c>
-      <c r="L687" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M687" t="str">
-        <v>07:51</v>
-      </c>
-      <c r="N687">
-        <v>93</v>
-      </c>
-      <c r="O687" t="str">
-        <v/>
-      </c>
-      <c r="P687" t="str">
-        <v/>
-      </c>
-      <c r="Q687" t="str">
-        <v/>
-      </c>
-      <c r="R687">
-        <v>93</v>
-      </c>
-      <c r="S687">
-        <v>93</v>
-      </c>
-      <c r="T687" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="688">
-      <c r="A688" t="str">
-        <v>1787221531088</v>
-      </c>
-      <c r="B688" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C688" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D688" t="str">
-        <v>m1026|||brown</v>
-      </c>
-      <c r="E688" t="str">
-        <v>M1026</v>
-      </c>
-      <c r="F688" t="str">
-        <v>BROWN</v>
-      </c>
-      <c r="G688" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H688" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I688" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J688" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K688" t="str">
-        <v/>
-      </c>
-      <c r="L688" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M688" t="str">
-        <v>07:51</v>
-      </c>
-      <c r="N688">
-        <v>167</v>
-      </c>
-      <c r="O688" t="str">
-        <v/>
-      </c>
-      <c r="P688" t="str">
-        <v/>
-      </c>
-      <c r="Q688" t="str">
-        <v/>
-      </c>
-      <c r="R688">
-        <v>167</v>
-      </c>
-      <c r="S688">
-        <v>175</v>
-      </c>
-      <c r="T688" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="689">
-      <c r="A689" t="str">
-        <v>1787221601849</v>
-      </c>
-      <c r="B689" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C689" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D689" t="str">
-        <v>m1012|||brown</v>
-      </c>
-      <c r="E689" t="str">
-        <v>M1012</v>
-      </c>
-      <c r="F689" t="str">
-        <v>BROWN</v>
-      </c>
-      <c r="G689" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H689" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I689" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J689" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K689" t="str">
-        <v/>
-      </c>
-      <c r="L689" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M689" t="str">
-        <v>07:51</v>
-      </c>
-      <c r="N689">
-        <v>457</v>
-      </c>
-      <c r="O689" t="str">
-        <v/>
-      </c>
-      <c r="P689" t="str">
-        <v/>
-      </c>
-      <c r="Q689" t="str">
-        <v/>
-      </c>
-      <c r="R689">
-        <v>457</v>
-      </c>
-      <c r="S689">
-        <v>457</v>
-      </c>
-      <c r="T689" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="690">
-      <c r="A690" t="str">
-        <v>1787221655193</v>
-      </c>
-      <c r="B690" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C690" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D690" t="str">
-        <v>m1034|||light wash</v>
-      </c>
-      <c r="E690" t="str">
-        <v>M1034</v>
-      </c>
-      <c r="F690" t="str">
-        <v>LIGHT WASH</v>
-      </c>
-      <c r="G690" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H690" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I690" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J690" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K690" t="str">
-        <v/>
-      </c>
-      <c r="L690" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M690" t="str">
-        <v>07:51</v>
-      </c>
-      <c r="N690">
-        <v>28</v>
-      </c>
-      <c r="O690" t="str">
-        <v/>
-      </c>
-      <c r="P690" t="str">
-        <v/>
-      </c>
-      <c r="Q690" t="str">
-        <v/>
-      </c>
-      <c r="R690">
-        <v>28</v>
-      </c>
-      <c r="S690">
-        <v>121</v>
-      </c>
-      <c r="T690" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="691">
-      <c r="A691" t="str">
-        <v>1787221707681</v>
-      </c>
-      <c r="B691" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C691" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D691" t="str">
-        <v>m1012|||sage brush</v>
-      </c>
-      <c r="E691" t="str">
-        <v>M1012</v>
-      </c>
-      <c r="F691" t="str">
-        <v>SAGE BRUSH</v>
-      </c>
-      <c r="G691" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H691" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I691" t="str">
-        <v>Pigment Dye</v>
-      </c>
-      <c r="J691" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K691" t="str">
-        <v>846</v>
-      </c>
-      <c r="L691" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M691" t="str">
-        <v>19:58</v>
-      </c>
-      <c r="N691">
-        <v>15</v>
-      </c>
-      <c r="O691" t="str">
-        <v/>
-      </c>
-      <c r="P691" t="str">
-        <v/>
-      </c>
-      <c r="Q691" t="str">
-        <v/>
-      </c>
-      <c r="R691">
-        <v>15</v>
-      </c>
-      <c r="S691">
-        <v>15</v>
-      </c>
-      <c r="T691" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="692">
-      <c r="A692" t="str">
-        <v>1787221759970</v>
-      </c>
-      <c r="B692" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C692" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D692" t="str">
-        <v>m1026|||olive green</v>
-      </c>
-      <c r="E692" t="str">
-        <v>M1026</v>
-      </c>
-      <c r="F692" t="str">
-        <v>OLIVE GREEN</v>
-      </c>
-      <c r="G692" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H692" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I692" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J692" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K692" t="str">
-        <v/>
-      </c>
-      <c r="L692" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M692" t="str">
-        <v>07:51</v>
-      </c>
-      <c r="N692">
-        <v>322</v>
-      </c>
-      <c r="O692" t="str">
-        <v/>
-      </c>
-      <c r="P692" t="str">
-        <v/>
-      </c>
-      <c r="Q692" t="str">
-        <v/>
-      </c>
-      <c r="R692">
-        <v>322</v>
-      </c>
-      <c r="S692">
-        <v>322</v>
-      </c>
-      <c r="T692" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="693">
-      <c r="A693" t="str">
-        <v>1787223356971</v>
-      </c>
-      <c r="B693" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C693" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D693" t="str">
-        <v>m1034|||medium wash</v>
-      </c>
-      <c r="E693" t="str">
-        <v>M1034</v>
-      </c>
-      <c r="F693" t="str">
-        <v>MEDIUM WASH</v>
-      </c>
-      <c r="G693" t="str">
-        <v>BDD</v>
-      </c>
-      <c r="H693" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I693" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J693" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K693" t="str">
-        <v/>
-      </c>
-      <c r="L693" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M693" t="str">
-        <v>07:51</v>
-      </c>
-      <c r="N693">
-        <v>16</v>
-      </c>
-      <c r="O693" t="str">
-        <v/>
-      </c>
-      <c r="P693" t="str">
-        <v/>
-      </c>
-      <c r="Q693" t="str">
-        <v/>
-      </c>
-      <c r="R693">
-        <v>16</v>
-      </c>
-      <c r="S693">
-        <v>16</v>
-      </c>
-      <c r="T693" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="694">
-      <c r="A694" t="str">
-        <v>1787223917363</v>
-      </c>
-      <c r="B694" t="str">
-        <v/>
-      </c>
-      <c r="C694" t="str">
-        <v/>
-      </c>
-      <c r="D694" t="str">
-        <v>20485245|||dark olive</v>
-      </c>
-      <c r="E694" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F694" t="str">
-        <v>DARK OLIVE</v>
-      </c>
-      <c r="G694" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H694" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I694" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J694" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K694" t="str">
-        <v/>
-      </c>
-      <c r="L694" t="str">
-        <v/>
-      </c>
-      <c r="M694" t="str">
-        <v>11:45</v>
-      </c>
-      <c r="N694">
-        <v>1</v>
-      </c>
-      <c r="O694" t="str">
-        <v/>
-      </c>
-      <c r="P694" t="str">
-        <v/>
-      </c>
-      <c r="Q694" t="str">
-        <v/>
-      </c>
-      <c r="R694">
-        <v>1</v>
-      </c>
-      <c r="S694">
-        <v>124</v>
-      </c>
-      <c r="T694" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="695">
-      <c r="A695" t="str">
-        <v>1787224044452</v>
-      </c>
-      <c r="B695" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C695" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D695" t="str">
-        <v>20485245|||dark navy</v>
-      </c>
-      <c r="E695" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F695" t="str">
-        <v>DARK NAVY</v>
-      </c>
-      <c r="G695" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H695" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I695" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J695" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K695" t="str">
-        <v/>
-      </c>
-      <c r="L695" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M695" t="str">
-        <v>11:45</v>
-      </c>
-      <c r="N695">
-        <v>51</v>
-      </c>
-      <c r="O695" t="str">
-        <v/>
-      </c>
-      <c r="P695" t="str">
-        <v/>
-      </c>
-      <c r="Q695" t="str">
-        <v/>
-      </c>
-      <c r="R695">
-        <v>51</v>
-      </c>
-      <c r="S695">
-        <v>51</v>
-      </c>
-      <c r="T695" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="696">
-      <c r="A696" t="str">
-        <v>1787224107876</v>
-      </c>
-      <c r="B696" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C696" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D696" t="str">
-        <v>20485245|||dark olive</v>
-      </c>
-      <c r="E696" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F696" t="str">
-        <v>DARK OLIVE</v>
-      </c>
-      <c r="G696" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H696" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I696" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J696" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K696" t="str">
-        <v/>
-      </c>
-      <c r="L696" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M696" t="str">
-        <v>08:15</v>
-      </c>
-      <c r="N696">
-        <v>2</v>
-      </c>
-      <c r="O696" t="str">
-        <v/>
-      </c>
-      <c r="P696" t="str">
-        <v/>
-      </c>
-      <c r="Q696" t="str">
-        <v/>
-      </c>
-      <c r="R696">
-        <v>2</v>
-      </c>
-      <c r="S696">
-        <v>126</v>
-      </c>
-      <c r="T696" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="697">
-      <c r="A697" t="str">
-        <v>1787224176381</v>
-      </c>
-      <c r="B697" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C697" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D697" t="str">
-        <v>20485245|||dark olive</v>
-      </c>
-      <c r="E697" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F697" t="str">
-        <v>DARK OLIVE</v>
-      </c>
-      <c r="G697" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H697" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I697" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J697" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K697" t="str">
-        <v/>
-      </c>
-      <c r="L697" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M697" t="str">
-        <v>08:39</v>
-      </c>
-      <c r="N697">
-        <v>15</v>
-      </c>
-      <c r="O697" t="str">
-        <v/>
-      </c>
-      <c r="P697" t="str">
-        <v/>
-      </c>
-      <c r="Q697" t="str">
-        <v/>
-      </c>
-      <c r="R697">
-        <v>15</v>
-      </c>
-      <c r="S697">
-        <v>141</v>
-      </c>
-      <c r="T697" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="698">
-      <c r="A698" t="str">
-        <v>1787224318038</v>
-      </c>
-      <c r="B698" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C698" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D698" t="str">
-        <v>20485245|||dark navy</v>
-      </c>
-      <c r="E698" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F698" t="str">
-        <v>DARK NAVY</v>
-      </c>
-      <c r="G698" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H698" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I698" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J698" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K698" t="str">
-        <v/>
-      </c>
-      <c r="L698" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M698" t="str">
-        <v>08:29</v>
-      </c>
-      <c r="N698">
-        <v>30</v>
-      </c>
-      <c r="O698" t="str">
-        <v/>
-      </c>
-      <c r="P698" t="str">
-        <v/>
-      </c>
-      <c r="Q698" t="str">
-        <v/>
-      </c>
-      <c r="R698">
-        <v>30</v>
-      </c>
-      <c r="S698">
-        <v>81</v>
-      </c>
-      <c r="T698" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="699">
-      <c r="A699" t="str">
-        <v>1787224420567</v>
-      </c>
-      <c r="B699" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C699" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D699" t="str">
-        <v>20485245|||dark olive</v>
-      </c>
-      <c r="E699" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F699" t="str">
-        <v>DARK OLIVE</v>
-      </c>
-      <c r="G699" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H699" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I699" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J699" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K699" t="str">
-        <v/>
-      </c>
-      <c r="L699" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M699" t="str">
-        <v>15:45</v>
-      </c>
-      <c r="N699">
-        <v>40</v>
-      </c>
-      <c r="O699" t="str">
-        <v/>
-      </c>
-      <c r="P699" t="str">
-        <v/>
-      </c>
-      <c r="Q699" t="str">
-        <v/>
-      </c>
-      <c r="R699">
-        <v>40</v>
-      </c>
-      <c r="S699">
-        <v>181</v>
-      </c>
-      <c r="T699" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="700">
-      <c r="A700" t="str">
-        <v>1787224711624</v>
-      </c>
-      <c r="B700" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C700" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D700" t="str">
-        <v>20485245|||dark olive</v>
-      </c>
-      <c r="E700" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F700" t="str">
-        <v>DARK OLIVE</v>
-      </c>
-      <c r="G700" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H700" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I700" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J700" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K700" t="str">
-        <v/>
-      </c>
-      <c r="L700" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M700" t="str">
-        <v>08:50</v>
-      </c>
-      <c r="N700">
-        <v>61</v>
-      </c>
-      <c r="O700" t="str">
-        <v/>
-      </c>
-      <c r="P700" t="str">
-        <v/>
-      </c>
-      <c r="Q700" t="str">
-        <v/>
-      </c>
-      <c r="R700">
-        <v>61</v>
-      </c>
-      <c r="S700">
-        <v>242</v>
-      </c>
-      <c r="T700" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="701">
-      <c r="A701" t="str">
-        <v>1787224794289</v>
-      </c>
-      <c r="B701" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C701" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D701" t="str">
-        <v>20485245|||dark olive</v>
-      </c>
-      <c r="E701" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F701" t="str">
-        <v>DARK OLIVE</v>
-      </c>
-      <c r="G701" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H701" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I701" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J701" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K701" t="str">
-        <v/>
-      </c>
-      <c r="L701" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M701" t="str">
-        <v>12:50</v>
-      </c>
-      <c r="N701">
-        <v>81</v>
-      </c>
-      <c r="O701" t="str">
-        <v/>
-      </c>
-      <c r="P701" t="str">
-        <v/>
-      </c>
-      <c r="Q701" t="str">
-        <v/>
-      </c>
-      <c r="R701">
-        <v>81</v>
-      </c>
-      <c r="S701">
-        <v>323</v>
-      </c>
-      <c r="T701" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="702">
-      <c r="A702" t="str">
-        <v>1787225046418</v>
-      </c>
-      <c r="B702" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C702" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D702" t="str">
-        <v>20485245|||dark navy</v>
-      </c>
-      <c r="E702" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F702" t="str">
-        <v>DARK NAVY</v>
-      </c>
-      <c r="G702" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H702" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I702" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J702" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K702" t="str">
-        <v/>
-      </c>
-      <c r="L702" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M702" t="str">
-        <v>13:53</v>
-      </c>
-      <c r="N702">
-        <v>71</v>
-      </c>
-      <c r="O702" t="str">
-        <v/>
-      </c>
-      <c r="P702" t="str">
-        <v/>
-      </c>
-      <c r="Q702" t="str">
-        <v/>
-      </c>
-      <c r="R702">
-        <v>71</v>
-      </c>
-      <c r="S702">
-        <v>152</v>
-      </c>
-      <c r="T702" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="703">
-      <c r="A703" t="str">
-        <v>1787225472831</v>
-      </c>
-      <c r="B703" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C703" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D703" t="str">
-        <v>20485245|||dark navy</v>
-      </c>
-      <c r="E703" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F703" t="str">
-        <v>DARK NAVY</v>
-      </c>
-      <c r="G703" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H703" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I703" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J703" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K703" t="str">
-        <v/>
-      </c>
-      <c r="L703" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M703" t="str">
-        <v>15:55</v>
-      </c>
-      <c r="N703">
-        <v>41</v>
-      </c>
-      <c r="O703" t="str">
-        <v/>
-      </c>
-      <c r="P703" t="str">
-        <v/>
-      </c>
-      <c r="Q703" t="str">
-        <v/>
-      </c>
-      <c r="R703">
-        <v>41</v>
-      </c>
-      <c r="S703">
-        <v>193</v>
-      </c>
-      <c r="T703" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T703"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T684"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -91017,16 +89839,16 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="Q2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="R2" t="str">
         <v>0</v>

</xml_diff>

<commit_message>
Emergency restore — blocking old app saves
</commit_message>
<xml_diff>
--- a/finishing_data.xlsx
+++ b/finishing_data.xlsx
@@ -515,7 +515,7 @@
         <v/>
       </c>
       <c r="J2" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K2" t="str">
         <v>No</v>
@@ -524,11 +524,11 @@
         <v>No</v>
       </c>
       <c r="M2" t="str">
+        <v>No</v>
+      </c>
+      <c r="N2" t="str">
         <v>3</v>
       </c>
-      <c r="N2" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O2" t="str">
         <v>Yes</v>
       </c>
@@ -542,19 +542,19 @@
         <v>Yes</v>
       </c>
       <c r="S2" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T2" t="str">
         <v>No</v>
       </c>
       <c r="U2" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W2" t="str">
         <v>6</v>
-      </c>
-      <c r="W2" t="str">
-        <v>0</v>
       </c>
       <c r="X2" t="str">
         <v>0</v>
@@ -598,7 +598,7 @@
         <v/>
       </c>
       <c r="J3" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K3" t="str">
         <v>No</v>
@@ -607,11 +607,11 @@
         <v>No</v>
       </c>
       <c r="M3" t="str">
+        <v>No</v>
+      </c>
+      <c r="N3" t="str">
         <v>3</v>
       </c>
-      <c r="N3" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O3" t="str">
         <v>Yes</v>
       </c>
@@ -625,19 +625,19 @@
         <v>Yes</v>
       </c>
       <c r="S3" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T3" t="str">
         <v>No</v>
       </c>
       <c r="U3" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V3" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W3" t="str">
         <v>6</v>
-      </c>
-      <c r="W3" t="str">
-        <v>0</v>
       </c>
       <c r="X3" t="str">
         <v>0</v>
@@ -681,7 +681,7 @@
         <v/>
       </c>
       <c r="J4" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K4" t="str">
         <v>No</v>
@@ -690,11 +690,11 @@
         <v>No</v>
       </c>
       <c r="M4" t="str">
+        <v>No</v>
+      </c>
+      <c r="N4" t="str">
         <v>3</v>
       </c>
-      <c r="N4" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O4" t="str">
         <v>Yes</v>
       </c>
@@ -708,19 +708,19 @@
         <v>Yes</v>
       </c>
       <c r="S4" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T4" t="str">
         <v>No</v>
       </c>
       <c r="U4" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V4" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W4" t="str">
         <v>6</v>
-      </c>
-      <c r="W4" t="str">
-        <v>0</v>
       </c>
       <c r="X4" t="str">
         <v>0</v>
@@ -764,7 +764,7 @@
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K5" t="str">
         <v>No</v>
@@ -773,11 +773,11 @@
         <v>No</v>
       </c>
       <c r="M5" t="str">
+        <v>No</v>
+      </c>
+      <c r="N5" t="str">
         <v>3</v>
       </c>
-      <c r="N5" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O5" t="str">
         <v>Yes</v>
       </c>
@@ -791,19 +791,19 @@
         <v>Yes</v>
       </c>
       <c r="S5" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T5" t="str">
         <v>No</v>
       </c>
       <c r="U5" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V5" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W5" t="str">
         <v>6</v>
-      </c>
-      <c r="W5" t="str">
-        <v>0</v>
       </c>
       <c r="X5" t="str">
         <v>0</v>
@@ -847,7 +847,7 @@
         <v/>
       </c>
       <c r="J6" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K6" t="str">
         <v>No</v>
@@ -856,11 +856,11 @@
         <v>No</v>
       </c>
       <c r="M6" t="str">
+        <v>No</v>
+      </c>
+      <c r="N6" t="str">
         <v>3</v>
       </c>
-      <c r="N6" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O6" t="str">
         <v>Yes</v>
       </c>
@@ -874,19 +874,19 @@
         <v>Yes</v>
       </c>
       <c r="S6" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T6" t="str">
         <v>No</v>
       </c>
       <c r="U6" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W6" t="str">
         <v>6</v>
-      </c>
-      <c r="W6" t="str">
-        <v>0</v>
       </c>
       <c r="X6" t="str">
         <v>0</v>
@@ -930,7 +930,7 @@
         <v/>
       </c>
       <c r="J7" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K7" t="str">
         <v>No</v>
@@ -939,11 +939,11 @@
         <v>No</v>
       </c>
       <c r="M7" t="str">
+        <v>No</v>
+      </c>
+      <c r="N7" t="str">
         <v>3</v>
       </c>
-      <c r="N7" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O7" t="str">
         <v>Yes</v>
       </c>
@@ -957,19 +957,19 @@
         <v>Yes</v>
       </c>
       <c r="S7" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T7" t="str">
         <v>No</v>
       </c>
       <c r="U7" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V7" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W7" t="str">
         <v>6</v>
-      </c>
-      <c r="W7" t="str">
-        <v>0</v>
       </c>
       <c r="X7" t="str">
         <v>0</v>
@@ -1013,7 +1013,7 @@
         <v/>
       </c>
       <c r="J8" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K8" t="str">
         <v>No</v>
@@ -1022,11 +1022,11 @@
         <v>No</v>
       </c>
       <c r="M8" t="str">
+        <v>No</v>
+      </c>
+      <c r="N8" t="str">
         <v>3</v>
       </c>
-      <c r="N8" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O8" t="str">
         <v>Yes</v>
       </c>
@@ -1040,19 +1040,19 @@
         <v>Yes</v>
       </c>
       <c r="S8" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T8" t="str">
         <v>No</v>
       </c>
       <c r="U8" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W8" t="str">
         <v>6</v>
-      </c>
-      <c r="W8" t="str">
-        <v>0</v>
       </c>
       <c r="X8" t="str">
         <v>0</v>
@@ -1096,7 +1096,7 @@
         <v/>
       </c>
       <c r="J9" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K9" t="str">
         <v>No</v>
@@ -1105,11 +1105,11 @@
         <v>No</v>
       </c>
       <c r="M9" t="str">
+        <v>No</v>
+      </c>
+      <c r="N9" t="str">
         <v>3</v>
       </c>
-      <c r="N9" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O9" t="str">
         <v>Yes</v>
       </c>
@@ -1123,19 +1123,19 @@
         <v>Yes</v>
       </c>
       <c r="S9" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T9" t="str">
         <v>No</v>
       </c>
       <c r="U9" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W9" t="str">
         <v>6</v>
-      </c>
-      <c r="W9" t="str">
-        <v>0</v>
       </c>
       <c r="X9" t="str">
         <v>0</v>
@@ -1179,7 +1179,7 @@
         <v/>
       </c>
       <c r="J10" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K10" t="str">
         <v>No</v>
@@ -1188,11 +1188,11 @@
         <v>No</v>
       </c>
       <c r="M10" t="str">
+        <v>No</v>
+      </c>
+      <c r="N10" t="str">
         <v>3</v>
       </c>
-      <c r="N10" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O10" t="str">
         <v>Yes</v>
       </c>
@@ -1206,19 +1206,19 @@
         <v>Yes</v>
       </c>
       <c r="S10" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T10" t="str">
         <v>No</v>
       </c>
       <c r="U10" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W10" t="str">
         <v>6</v>
-      </c>
-      <c r="W10" t="str">
-        <v>0</v>
       </c>
       <c r="X10" t="str">
         <v>0</v>
@@ -1262,7 +1262,7 @@
         <v/>
       </c>
       <c r="J11" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K11" t="str">
         <v>No</v>
@@ -1271,11 +1271,11 @@
         <v>No</v>
       </c>
       <c r="M11" t="str">
+        <v>No</v>
+      </c>
+      <c r="N11" t="str">
         <v>3</v>
       </c>
-      <c r="N11" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O11" t="str">
         <v>Yes</v>
       </c>
@@ -1289,19 +1289,19 @@
         <v>Yes</v>
       </c>
       <c r="S11" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T11" t="str">
         <v>No</v>
       </c>
       <c r="U11" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V11" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W11" t="str">
         <v>6</v>
-      </c>
-      <c r="W11" t="str">
-        <v>0</v>
       </c>
       <c r="X11" t="str">
         <v>0</v>
@@ -1345,7 +1345,7 @@
         <v/>
       </c>
       <c r="J12" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K12" t="str">
         <v>No</v>
@@ -1354,11 +1354,11 @@
         <v>No</v>
       </c>
       <c r="M12" t="str">
+        <v>No</v>
+      </c>
+      <c r="N12" t="str">
         <v>3</v>
       </c>
-      <c r="N12" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O12" t="str">
         <v>Yes</v>
       </c>
@@ -1372,19 +1372,19 @@
         <v>Yes</v>
       </c>
       <c r="S12" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T12" t="str">
         <v>No</v>
       </c>
       <c r="U12" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W12" t="str">
         <v>6</v>
-      </c>
-      <c r="W12" t="str">
-        <v>0</v>
       </c>
       <c r="X12" t="str">
         <v>0</v>
@@ -1428,7 +1428,7 @@
         <v/>
       </c>
       <c r="J13" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K13" t="str">
         <v>No</v>
@@ -1437,11 +1437,11 @@
         <v>No</v>
       </c>
       <c r="M13" t="str">
+        <v>No</v>
+      </c>
+      <c r="N13" t="str">
         <v>3</v>
       </c>
-      <c r="N13" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O13" t="str">
         <v>Yes</v>
       </c>
@@ -1455,19 +1455,19 @@
         <v>Yes</v>
       </c>
       <c r="S13" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T13" t="str">
         <v>No</v>
       </c>
       <c r="U13" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W13" t="str">
         <v>6</v>
-      </c>
-      <c r="W13" t="str">
-        <v>0</v>
       </c>
       <c r="X13" t="str">
         <v>0</v>
@@ -1511,7 +1511,7 @@
         <v/>
       </c>
       <c r="J14" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K14" t="str">
         <v>No</v>
@@ -1520,11 +1520,11 @@
         <v>No</v>
       </c>
       <c r="M14" t="str">
+        <v>No</v>
+      </c>
+      <c r="N14" t="str">
         <v>3</v>
       </c>
-      <c r="N14" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O14" t="str">
         <v>Yes</v>
       </c>
@@ -1538,19 +1538,19 @@
         <v>Yes</v>
       </c>
       <c r="S14" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T14" t="str">
         <v>No</v>
       </c>
       <c r="U14" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V14" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W14" t="str">
         <v>6</v>
-      </c>
-      <c r="W14" t="str">
-        <v>0</v>
       </c>
       <c r="X14" t="str">
         <v>0</v>
@@ -1594,7 +1594,7 @@
         <v/>
       </c>
       <c r="J15" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K15" t="str">
         <v>No</v>
@@ -1603,11 +1603,11 @@
         <v>No</v>
       </c>
       <c r="M15" t="str">
+        <v>No</v>
+      </c>
+      <c r="N15" t="str">
         <v>3</v>
       </c>
-      <c r="N15" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O15" t="str">
         <v>Yes</v>
       </c>
@@ -1621,19 +1621,19 @@
         <v>Yes</v>
       </c>
       <c r="S15" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T15" t="str">
         <v>No</v>
       </c>
       <c r="U15" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V15" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W15" t="str">
         <v>6</v>
-      </c>
-      <c r="W15" t="str">
-        <v>0</v>
       </c>
       <c r="X15" t="str">
         <v>0</v>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J16" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K16" t="str">
         <v>No</v>
@@ -1686,11 +1686,11 @@
         <v>No</v>
       </c>
       <c r="M16" t="str">
+        <v>No</v>
+      </c>
+      <c r="N16" t="str">
         <v>3</v>
       </c>
-      <c r="N16" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O16" t="str">
         <v>Yes</v>
       </c>
@@ -1704,19 +1704,19 @@
         <v>Yes</v>
       </c>
       <c r="S16" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T16" t="str">
         <v>No</v>
       </c>
       <c r="U16" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V16" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W16" t="str">
         <v>6</v>
-      </c>
-      <c r="W16" t="str">
-        <v>0</v>
       </c>
       <c r="X16" t="str">
         <v>0</v>
@@ -1760,7 +1760,7 @@
         <v/>
       </c>
       <c r="J17" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K17" t="str">
         <v>No</v>
@@ -1769,11 +1769,11 @@
         <v>No</v>
       </c>
       <c r="M17" t="str">
+        <v>No</v>
+      </c>
+      <c r="N17" t="str">
         <v>3</v>
       </c>
-      <c r="N17" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O17" t="str">
         <v>Yes</v>
       </c>
@@ -1787,19 +1787,19 @@
         <v>Yes</v>
       </c>
       <c r="S17" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T17" t="str">
         <v>No</v>
       </c>
       <c r="U17" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W17" t="str">
         <v>6</v>
-      </c>
-      <c r="W17" t="str">
-        <v>0</v>
       </c>
       <c r="X17" t="str">
         <v>0</v>
@@ -1843,7 +1843,7 @@
         <v/>
       </c>
       <c r="J18" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K18" t="str">
         <v>No</v>
@@ -1852,11 +1852,11 @@
         <v>No</v>
       </c>
       <c r="M18" t="str">
+        <v>No</v>
+      </c>
+      <c r="N18" t="str">
         <v>3</v>
       </c>
-      <c r="N18" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O18" t="str">
         <v>Yes</v>
       </c>
@@ -1870,19 +1870,19 @@
         <v>Yes</v>
       </c>
       <c r="S18" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T18" t="str">
         <v>No</v>
       </c>
       <c r="U18" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W18" t="str">
         <v>6</v>
-      </c>
-      <c r="W18" t="str">
-        <v>0</v>
       </c>
       <c r="X18" t="str">
         <v>0</v>
@@ -1926,7 +1926,7 @@
         <v/>
       </c>
       <c r="J19" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K19" t="str">
         <v>No</v>
@@ -1935,11 +1935,11 @@
         <v>No</v>
       </c>
       <c r="M19" t="str">
+        <v>No</v>
+      </c>
+      <c r="N19" t="str">
         <v>3</v>
       </c>
-      <c r="N19" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O19" t="str">
         <v>Yes</v>
       </c>
@@ -1953,19 +1953,19 @@
         <v>Yes</v>
       </c>
       <c r="S19" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T19" t="str">
         <v>No</v>
       </c>
       <c r="U19" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W19" t="str">
         <v>6</v>
-      </c>
-      <c r="W19" t="str">
-        <v>0</v>
       </c>
       <c r="X19" t="str">
         <v>0</v>
@@ -2009,7 +2009,7 @@
         <v/>
       </c>
       <c r="J20" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K20" t="str">
         <v>No</v>
@@ -2018,11 +2018,11 @@
         <v>No</v>
       </c>
       <c r="M20" t="str">
+        <v>No</v>
+      </c>
+      <c r="N20" t="str">
         <v>3</v>
       </c>
-      <c r="N20" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O20" t="str">
         <v>Yes</v>
       </c>
@@ -2036,19 +2036,19 @@
         <v>Yes</v>
       </c>
       <c r="S20" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T20" t="str">
         <v>No</v>
       </c>
       <c r="U20" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W20" t="str">
         <v>6</v>
-      </c>
-      <c r="W20" t="str">
-        <v>0</v>
       </c>
       <c r="X20" t="str">
         <v>0</v>
@@ -2092,7 +2092,7 @@
         <v/>
       </c>
       <c r="J21" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K21" t="str">
         <v>No</v>
@@ -2101,11 +2101,11 @@
         <v>No</v>
       </c>
       <c r="M21" t="str">
+        <v>No</v>
+      </c>
+      <c r="N21" t="str">
         <v>3</v>
       </c>
-      <c r="N21" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O21" t="str">
         <v>Yes</v>
       </c>
@@ -2119,19 +2119,19 @@
         <v>Yes</v>
       </c>
       <c r="S21" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T21" t="str">
         <v>No</v>
       </c>
       <c r="U21" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W21" t="str">
         <v>6</v>
-      </c>
-      <c r="W21" t="str">
-        <v>0</v>
       </c>
       <c r="X21" t="str">
         <v>0</v>
@@ -2175,7 +2175,7 @@
         <v/>
       </c>
       <c r="J22" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K22" t="str">
         <v>No</v>
@@ -2184,11 +2184,11 @@
         <v>No</v>
       </c>
       <c r="M22" t="str">
+        <v>No</v>
+      </c>
+      <c r="N22" t="str">
         <v>3</v>
       </c>
-      <c r="N22" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O22" t="str">
         <v>Yes</v>
       </c>
@@ -2202,19 +2202,19 @@
         <v>Yes</v>
       </c>
       <c r="S22" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T22" t="str">
         <v>No</v>
       </c>
       <c r="U22" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V22" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W22" t="str">
         <v>6</v>
-      </c>
-      <c r="W22" t="str">
-        <v>0</v>
       </c>
       <c r="X22" t="str">
         <v>0</v>
@@ -2258,7 +2258,7 @@
         <v/>
       </c>
       <c r="J23" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K23" t="str">
         <v>No</v>
@@ -2267,11 +2267,11 @@
         <v>No</v>
       </c>
       <c r="M23" t="str">
+        <v>No</v>
+      </c>
+      <c r="N23" t="str">
         <v>3</v>
       </c>
-      <c r="N23" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O23" t="str">
         <v>Yes</v>
       </c>
@@ -2285,19 +2285,19 @@
         <v>Yes</v>
       </c>
       <c r="S23" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T23" t="str">
         <v>No</v>
       </c>
       <c r="U23" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V23" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W23" t="str">
         <v>6</v>
-      </c>
-      <c r="W23" t="str">
-        <v>0</v>
       </c>
       <c r="X23" t="str">
         <v>0</v>
@@ -2341,7 +2341,7 @@
         <v/>
       </c>
       <c r="J24" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K24" t="str">
         <v>No</v>
@@ -2350,11 +2350,11 @@
         <v>No</v>
       </c>
       <c r="M24" t="str">
+        <v>No</v>
+      </c>
+      <c r="N24" t="str">
         <v>3</v>
       </c>
-      <c r="N24" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O24" t="str">
         <v>Yes</v>
       </c>
@@ -2368,19 +2368,19 @@
         <v>Yes</v>
       </c>
       <c r="S24" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T24" t="str">
         <v>No</v>
       </c>
       <c r="U24" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V24" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W24" t="str">
         <v>6</v>
-      </c>
-      <c r="W24" t="str">
-        <v>0</v>
       </c>
       <c r="X24" t="str">
         <v>0</v>
@@ -2424,7 +2424,7 @@
         <v/>
       </c>
       <c r="J25" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K25" t="str">
         <v>No</v>
@@ -2433,11 +2433,11 @@
         <v>No</v>
       </c>
       <c r="M25" t="str">
+        <v>No</v>
+      </c>
+      <c r="N25" t="str">
         <v>3</v>
       </c>
-      <c r="N25" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O25" t="str">
         <v>Yes</v>
       </c>
@@ -2451,19 +2451,19 @@
         <v>Yes</v>
       </c>
       <c r="S25" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T25" t="str">
         <v>No</v>
       </c>
       <c r="U25" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V25" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W25" t="str">
         <v>6</v>
-      </c>
-      <c r="W25" t="str">
-        <v>0</v>
       </c>
       <c r="X25" t="str">
         <v>0</v>
@@ -2507,7 +2507,7 @@
         <v/>
       </c>
       <c r="J26" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K26" t="str">
         <v>No</v>
@@ -2516,11 +2516,11 @@
         <v>No</v>
       </c>
       <c r="M26" t="str">
+        <v>No</v>
+      </c>
+      <c r="N26" t="str">
         <v>3</v>
       </c>
-      <c r="N26" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O26" t="str">
         <v>Yes</v>
       </c>
@@ -2534,19 +2534,19 @@
         <v>Yes</v>
       </c>
       <c r="S26" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T26" t="str">
         <v>No</v>
       </c>
       <c r="U26" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V26" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W26" t="str">
         <v>6</v>
-      </c>
-      <c r="W26" t="str">
-        <v>0</v>
       </c>
       <c r="X26" t="str">
         <v>0</v>
@@ -2590,7 +2590,7 @@
         <v/>
       </c>
       <c r="J27" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K27" t="str">
         <v>No</v>
@@ -2599,11 +2599,11 @@
         <v>No</v>
       </c>
       <c r="M27" t="str">
+        <v>No</v>
+      </c>
+      <c r="N27" t="str">
         <v>3</v>
       </c>
-      <c r="N27" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O27" t="str">
         <v>Yes</v>
       </c>
@@ -2617,19 +2617,19 @@
         <v>Yes</v>
       </c>
       <c r="S27" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T27" t="str">
         <v>No</v>
       </c>
       <c r="U27" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V27" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W27" t="str">
         <v>6</v>
-      </c>
-      <c r="W27" t="str">
-        <v>0</v>
       </c>
       <c r="X27" t="str">
         <v>0</v>
@@ -2673,7 +2673,7 @@
         <v/>
       </c>
       <c r="J28" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K28" t="str">
         <v>No</v>
@@ -2682,11 +2682,11 @@
         <v>No</v>
       </c>
       <c r="M28" t="str">
+        <v>No</v>
+      </c>
+      <c r="N28" t="str">
         <v>3</v>
       </c>
-      <c r="N28" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O28" t="str">
         <v>Yes</v>
       </c>
@@ -2700,19 +2700,19 @@
         <v>Yes</v>
       </c>
       <c r="S28" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T28" t="str">
         <v>No</v>
       </c>
       <c r="U28" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V28" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W28" t="str">
         <v>6</v>
-      </c>
-      <c r="W28" t="str">
-        <v>0</v>
       </c>
       <c r="X28" t="str">
         <v>0</v>
@@ -2756,7 +2756,7 @@
         <v/>
       </c>
       <c r="J29" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K29" t="str">
         <v>No</v>
@@ -2765,11 +2765,11 @@
         <v>No</v>
       </c>
       <c r="M29" t="str">
+        <v>No</v>
+      </c>
+      <c r="N29" t="str">
         <v>3</v>
       </c>
-      <c r="N29" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O29" t="str">
         <v>Yes</v>
       </c>
@@ -2783,19 +2783,19 @@
         <v>Yes</v>
       </c>
       <c r="S29" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T29" t="str">
         <v>No</v>
       </c>
       <c r="U29" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V29" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W29" t="str">
         <v>6</v>
-      </c>
-      <c r="W29" t="str">
-        <v>0</v>
       </c>
       <c r="X29" t="str">
         <v>0</v>
@@ -2839,7 +2839,7 @@
         <v/>
       </c>
       <c r="J30" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K30" t="str">
         <v>No</v>
@@ -2848,11 +2848,11 @@
         <v>No</v>
       </c>
       <c r="M30" t="str">
+        <v>No</v>
+      </c>
+      <c r="N30" t="str">
         <v>3</v>
       </c>
-      <c r="N30" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O30" t="str">
         <v>Yes</v>
       </c>
@@ -2866,19 +2866,19 @@
         <v>Yes</v>
       </c>
       <c r="S30" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T30" t="str">
         <v>No</v>
       </c>
       <c r="U30" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V30" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W30" t="str">
         <v>6</v>
-      </c>
-      <c r="W30" t="str">
-        <v>0</v>
       </c>
       <c r="X30" t="str">
         <v>0</v>
@@ -2922,7 +2922,7 @@
         <v/>
       </c>
       <c r="J31" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K31" t="str">
         <v>No</v>
@@ -2931,11 +2931,11 @@
         <v>No</v>
       </c>
       <c r="M31" t="str">
+        <v>No</v>
+      </c>
+      <c r="N31" t="str">
         <v>3</v>
       </c>
-      <c r="N31" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O31" t="str">
         <v>Yes</v>
       </c>
@@ -2949,19 +2949,19 @@
         <v>Yes</v>
       </c>
       <c r="S31" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T31" t="str">
         <v>No</v>
       </c>
       <c r="U31" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V31" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W31" t="str">
         <v>6</v>
-      </c>
-      <c r="W31" t="str">
-        <v>0</v>
       </c>
       <c r="X31" t="str">
         <v>0</v>
@@ -3005,7 +3005,7 @@
         <v/>
       </c>
       <c r="J32" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K32" t="str">
         <v>No</v>
@@ -3014,11 +3014,11 @@
         <v>No</v>
       </c>
       <c r="M32" t="str">
+        <v>No</v>
+      </c>
+      <c r="N32" t="str">
         <v>3</v>
       </c>
-      <c r="N32" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O32" t="str">
         <v>Yes</v>
       </c>
@@ -3032,19 +3032,19 @@
         <v>Yes</v>
       </c>
       <c r="S32" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T32" t="str">
         <v>No</v>
       </c>
       <c r="U32" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V32" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W32" t="str">
         <v>6</v>
-      </c>
-      <c r="W32" t="str">
-        <v>0</v>
       </c>
       <c r="X32" t="str">
         <v>0</v>
@@ -3088,7 +3088,7 @@
         <v/>
       </c>
       <c r="J33" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K33" t="str">
         <v>No</v>
@@ -3097,11 +3097,11 @@
         <v>No</v>
       </c>
       <c r="M33" t="str">
+        <v>No</v>
+      </c>
+      <c r="N33" t="str">
         <v>3</v>
       </c>
-      <c r="N33" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O33" t="str">
         <v>Yes</v>
       </c>
@@ -3115,19 +3115,19 @@
         <v>Yes</v>
       </c>
       <c r="S33" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T33" t="str">
         <v>No</v>
       </c>
       <c r="U33" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V33" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W33" t="str">
         <v>6</v>
-      </c>
-      <c r="W33" t="str">
-        <v>0</v>
       </c>
       <c r="X33" t="str">
         <v>0</v>
@@ -3171,7 +3171,7 @@
         <v/>
       </c>
       <c r="J34" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K34" t="str">
         <v>No</v>
@@ -3180,11 +3180,11 @@
         <v>No</v>
       </c>
       <c r="M34" t="str">
+        <v>No</v>
+      </c>
+      <c r="N34" t="str">
         <v>3</v>
       </c>
-      <c r="N34" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O34" t="str">
         <v>Yes</v>
       </c>
@@ -3198,19 +3198,19 @@
         <v>Yes</v>
       </c>
       <c r="S34" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T34" t="str">
         <v>No</v>
       </c>
       <c r="U34" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V34" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W34" t="str">
         <v>6</v>
-      </c>
-      <c r="W34" t="str">
-        <v>0</v>
       </c>
       <c r="X34" t="str">
         <v>0</v>
@@ -3254,7 +3254,7 @@
         <v/>
       </c>
       <c r="J35" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="K35" t="str">
         <v>No</v>
@@ -3263,11 +3263,11 @@
         <v>No</v>
       </c>
       <c r="M35" t="str">
+        <v>No</v>
+      </c>
+      <c r="N35" t="str">
         <v>3</v>
       </c>
-      <c r="N35" t="str">
-        <v>Yes</v>
-      </c>
       <c r="O35" t="str">
         <v>Yes</v>
       </c>
@@ -3281,19 +3281,19 @@
         <v>Yes</v>
       </c>
       <c r="S35" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="T35" t="str">
         <v>No</v>
       </c>
       <c r="U35" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V35" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="W35" t="str">
         <v>6</v>
-      </c>
-      <c r="W35" t="str">
-        <v>0</v>
       </c>
       <c r="X35" t="str">
         <v>0</v>
@@ -3317,7 +3317,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T695"/>
+  <dimension ref="A1:T685"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -45729,7 +45729,7 @@
     </row>
     <row r="685">
       <c r="A685" t="str">
-        <v>1787235443859</v>
+        <v>1787227068567</v>
       </c>
       <c r="B685" t="str">
         <v>Aug 2026</v>
@@ -45738,13 +45738,13 @@
         <v>W34</v>
       </c>
       <c r="D685" t="str">
-        <v>20485245|||dark olive</v>
+        <v>20485245|||dark navy</v>
       </c>
       <c r="E685" t="str">
         <v>20485245</v>
       </c>
       <c r="F685" t="str">
-        <v>DARK OLIVE</v>
+        <v>DARK NAVY</v>
       </c>
       <c r="G685" t="str">
         <v>SGL</v>
@@ -45762,13 +45762,13 @@
         <v/>
       </c>
       <c r="L685" t="str">
-        <v>2026-08-19</v>
+        <v>2026-08-20</v>
       </c>
       <c r="M685" t="str">
-        <v>10:52</v>
+        <v>17:00</v>
       </c>
       <c r="N685">
-        <v>81</v>
+        <v>20</v>
       </c>
       <c r="O685" t="str">
         <v/>
@@ -45780,638 +45780,18 @@
         <v/>
       </c>
       <c r="R685">
-        <v>81</v>
+        <v>20</v>
       </c>
       <c r="S685">
-        <v>204</v>
+        <v>20</v>
       </c>
       <c r="T685" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="686">
-      <c r="A686" t="str">
-        <v>1787235487595</v>
-      </c>
-      <c r="B686" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C686" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D686" t="str">
-        <v>20485245|||dark olive</v>
-      </c>
-      <c r="E686" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F686" t="str">
-        <v>DARK OLIVE</v>
-      </c>
-      <c r="G686" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H686" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I686" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J686" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K686" t="str">
-        <v/>
-      </c>
-      <c r="L686" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M686" t="str">
-        <v>08:50</v>
-      </c>
-      <c r="N686">
-        <v>61</v>
-      </c>
-      <c r="O686" t="str">
-        <v/>
-      </c>
-      <c r="P686" t="str">
-        <v/>
-      </c>
-      <c r="Q686" t="str">
-        <v/>
-      </c>
-      <c r="R686">
-        <v>61</v>
-      </c>
-      <c r="S686">
-        <v>265</v>
-      </c>
-      <c r="T686" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="687">
-      <c r="A687" t="str">
-        <v>1787235508356</v>
-      </c>
-      <c r="B687" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C687" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D687" t="str">
-        <v>20485245|||dark olive</v>
-      </c>
-      <c r="E687" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F687" t="str">
-        <v>DARK OLIVE</v>
-      </c>
-      <c r="G687" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H687" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I687" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J687" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K687" t="str">
-        <v/>
-      </c>
-      <c r="L687" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M687" t="str">
-        <v>15:45</v>
-      </c>
-      <c r="N687">
-        <v>40</v>
-      </c>
-      <c r="O687" t="str">
-        <v/>
-      </c>
-      <c r="P687" t="str">
-        <v/>
-      </c>
-      <c r="Q687" t="str">
-        <v/>
-      </c>
-      <c r="R687">
-        <v>40</v>
-      </c>
-      <c r="S687">
-        <v>305</v>
-      </c>
-      <c r="T687" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="688">
-      <c r="A688" t="str">
-        <v>1787235536700</v>
-      </c>
-      <c r="B688" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C688" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D688" t="str">
-        <v>20485245|||dark olive</v>
-      </c>
-      <c r="E688" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F688" t="str">
-        <v>DARK OLIVE</v>
-      </c>
-      <c r="G688" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H688" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I688" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J688" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K688" t="str">
-        <v/>
-      </c>
-      <c r="L688" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M688" t="str">
-        <v>08:00</v>
-      </c>
-      <c r="N688">
-        <v>15</v>
-      </c>
-      <c r="O688" t="str">
-        <v/>
-      </c>
-      <c r="P688" t="str">
-        <v/>
-      </c>
-      <c r="Q688" t="str">
-        <v/>
-      </c>
-      <c r="R688">
-        <v>15</v>
-      </c>
-      <c r="S688">
-        <v>320</v>
-      </c>
-      <c r="T688" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="689">
-      <c r="A689" t="str">
-        <v>1787235551868</v>
-      </c>
-      <c r="B689" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C689" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D689" t="str">
-        <v>20485245|||dark navy</v>
-      </c>
-      <c r="E689" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F689" t="str">
-        <v>DARK NAVY</v>
-      </c>
-      <c r="G689" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H689" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I689" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J689" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K689" t="str">
-        <v/>
-      </c>
-      <c r="L689" t="str">
-        <v>2026-08-19</v>
-      </c>
-      <c r="M689" t="str">
-        <v>08:00</v>
-      </c>
-      <c r="N689">
-        <v>30</v>
-      </c>
-      <c r="O689" t="str">
-        <v/>
-      </c>
-      <c r="P689" t="str">
-        <v/>
-      </c>
-      <c r="Q689" t="str">
-        <v/>
-      </c>
-      <c r="R689">
-        <v>30</v>
-      </c>
-      <c r="S689">
-        <v>30</v>
-      </c>
-      <c r="T689" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="690">
-      <c r="A690" t="str">
-        <v>1787235567668</v>
-      </c>
-      <c r="B690" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C690" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D690" t="str">
-        <v>20485245|||dark navy</v>
-      </c>
-      <c r="E690" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F690" t="str">
-        <v>DARK NAVY</v>
-      </c>
-      <c r="G690" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H690" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I690" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J690" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K690" t="str">
-        <v/>
-      </c>
-      <c r="L690" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M690" t="str">
-        <v>10:55</v>
-      </c>
-      <c r="N690">
-        <v>71</v>
-      </c>
-      <c r="O690" t="str">
-        <v/>
-      </c>
-      <c r="P690" t="str">
-        <v/>
-      </c>
-      <c r="Q690" t="str">
-        <v/>
-      </c>
-      <c r="R690">
-        <v>71</v>
-      </c>
-      <c r="S690">
-        <v>101</v>
-      </c>
-      <c r="T690" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="691">
-      <c r="A691" t="str">
-        <v>1787235588244</v>
-      </c>
-      <c r="B691" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C691" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D691" t="str">
-        <v>20485245|||dark navy</v>
-      </c>
-      <c r="E691" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F691" t="str">
-        <v>DARK NAVY</v>
-      </c>
-      <c r="G691" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H691" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I691" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J691" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K691" t="str">
-        <v/>
-      </c>
-      <c r="L691" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M691" t="str">
-        <v>15:55</v>
-      </c>
-      <c r="N691">
-        <v>41</v>
-      </c>
-      <c r="O691" t="str">
-        <v/>
-      </c>
-      <c r="P691" t="str">
-        <v/>
-      </c>
-      <c r="Q691" t="str">
-        <v/>
-      </c>
-      <c r="R691">
-        <v>41</v>
-      </c>
-      <c r="S691">
-        <v>142</v>
-      </c>
-      <c r="T691" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="692">
-      <c r="A692" t="str">
-        <v>1787235601236</v>
-      </c>
-      <c r="B692" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C692" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D692" t="str">
-        <v>20485245|||dark olive</v>
-      </c>
-      <c r="E692" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F692" t="str">
-        <v>DARK OLIVE</v>
-      </c>
-      <c r="G692" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H692" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I692" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J692" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K692" t="str">
-        <v/>
-      </c>
-      <c r="L692" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M692" t="str">
-        <v>11:45</v>
-      </c>
-      <c r="N692">
-        <v>1</v>
-      </c>
-      <c r="O692" t="str">
-        <v/>
-      </c>
-      <c r="P692" t="str">
-        <v/>
-      </c>
-      <c r="Q692" t="str">
-        <v/>
-      </c>
-      <c r="R692">
-        <v>1</v>
-      </c>
-      <c r="S692">
-        <v>321</v>
-      </c>
-      <c r="T692" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="693">
-      <c r="A693" t="str">
-        <v>1787235624964</v>
-      </c>
-      <c r="B693" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C693" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D693" t="str">
-        <v>20485245|||dark olive</v>
-      </c>
-      <c r="E693" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F693" t="str">
-        <v>DARK OLIVE</v>
-      </c>
-      <c r="G693" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H693" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I693" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J693" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K693" t="str">
-        <v/>
-      </c>
-      <c r="L693" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M693" t="str">
-        <v>08:15</v>
-      </c>
-      <c r="N693">
-        <v>2</v>
-      </c>
-      <c r="O693" t="str">
-        <v/>
-      </c>
-      <c r="P693" t="str">
-        <v/>
-      </c>
-      <c r="Q693" t="str">
-        <v/>
-      </c>
-      <c r="R693">
-        <v>2</v>
-      </c>
-      <c r="S693">
-        <v>323</v>
-      </c>
-      <c r="T693" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="694">
-      <c r="A694" t="str">
-        <v>1787235646780</v>
-      </c>
-      <c r="B694" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C694" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D694" t="str">
-        <v>20485245|||dark navy</v>
-      </c>
-      <c r="E694" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F694" t="str">
-        <v>DARK NAVY</v>
-      </c>
-      <c r="G694" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H694" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I694" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J694" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K694" t="str">
-        <v/>
-      </c>
-      <c r="L694" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M694" t="str">
-        <v>17:00</v>
-      </c>
-      <c r="N694">
-        <v>20</v>
-      </c>
-      <c r="O694" t="str">
-        <v/>
-      </c>
-      <c r="P694" t="str">
-        <v/>
-      </c>
-      <c r="Q694" t="str">
-        <v/>
-      </c>
-      <c r="R694">
-        <v>20</v>
-      </c>
-      <c r="S694">
-        <v>162</v>
-      </c>
-      <c r="T694" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="695">
-      <c r="A695" t="str">
-        <v>1787235878054</v>
-      </c>
-      <c r="B695" t="str">
-        <v>Aug 2026</v>
-      </c>
-      <c r="C695" t="str">
-        <v>W34</v>
-      </c>
-      <c r="D695" t="str">
-        <v>20485245|||dark navy</v>
-      </c>
-      <c r="E695" t="str">
-        <v>20485245</v>
-      </c>
-      <c r="F695" t="str">
-        <v>DARK NAVY</v>
-      </c>
-      <c r="G695" t="str">
-        <v>SGL</v>
-      </c>
-      <c r="H695" t="str">
-        <v>Jkt</v>
-      </c>
-      <c r="I695" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="J695" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="K695" t="str">
-        <v/>
-      </c>
-      <c r="L695" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="M695" t="str">
-        <v>11:45</v>
-      </c>
-      <c r="N695">
-        <v>51</v>
-      </c>
-      <c r="O695" t="str">
-        <v/>
-      </c>
-      <c r="P695" t="str">
-        <v/>
-      </c>
-      <c r="Q695" t="str">
-        <v/>
-      </c>
-      <c r="R695">
-        <v>51</v>
-      </c>
-      <c r="S695">
-        <v>213</v>
-      </c>
-      <c r="T695" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T695"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T685"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -90515,22 +89895,22 @@
         <v>0</v>
       </c>
       <c r="L2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="Q2">
-        <v>NaN</v>
+        <v>0</v>
       </c>
       <c r="R2" t="str">
         <v>0</v>

</xml_diff>